<commit_message>
Atualizando a documentação do projeto integrador - 17/04/2026
</commit_message>
<xml_diff>
--- a/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/dicionario_de_dados_projeto.xlsx
+++ b/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/dicionario_de_dados_projeto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gusta\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aluno\Documents\Projetos_ADSN_Einstein\Terceiro_Semestre\Projeto_Integrador\Documentação\dicionario_dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83902419-7510-4827-AD41-28D29528E989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0911E6-20BD-4BF9-B7C3-EB184AF315FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{469F5BF7-1942-432A-8289-DDFBF75692AC}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -303,7 +301,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1077,71 +1075,71 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{064BA25E-541B-4771-AFA8-C0176CB4D374}">
   <dimension ref="A1:BT62"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.88671875" customWidth="1"/>
-    <col min="14" max="14" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.3984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.3984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.8984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.8984375" customWidth="1"/>
+    <col min="14" max="14" width="21.296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.09765625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.88671875" style="31"/>
-    <col min="26" max="26" width="20.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.69921875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.69921875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.8984375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25.09765625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.8984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.8984375" style="31"/>
+    <col min="26" max="26" width="20.296875" style="31" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="22" style="31" customWidth="1"/>
-    <col min="28" max="28" width="8.88671875" style="31"/>
-    <col min="29" max="29" width="14.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="30" max="32" width="8.88671875" style="31"/>
-    <col min="33" max="33" width="12.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.88671875" style="31" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8.88671875" style="31"/>
-    <col min="38" max="38" width="19.109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="26.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="42" max="44" width="8.88671875" style="31"/>
-    <col min="45" max="45" width="12.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="22.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.88671875" style="31" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="18.88671875" style="31" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.88671875" style="31"/>
-    <col min="50" max="50" width="18.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="22.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="8.88671875" style="31"/>
-    <col min="53" max="53" width="14.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="55" max="56" width="8.88671875" style="31"/>
-    <col min="57" max="57" width="12.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="22.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.88671875" style="31" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="20.109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="8.88671875" style="31"/>
-    <col min="62" max="62" width="18.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="22.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="8.88671875" style="31"/>
-    <col min="65" max="65" width="14.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="66" max="68" width="8.88671875" style="31"/>
-    <col min="69" max="69" width="12.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.88671875" style="31" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="16.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.8984375" style="31"/>
+    <col min="29" max="29" width="14.3984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="30" max="32" width="8.8984375" style="31"/>
+    <col min="33" max="33" width="12.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.09765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.8984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.69921875" style="31" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.8984375" style="31"/>
+    <col min="38" max="38" width="19.09765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="26.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.69921875" style="31" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="14.3984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="42" max="44" width="8.8984375" style="31"/>
+    <col min="45" max="45" width="12.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="22.69921875" style="31" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.8984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="18.8984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="8.8984375" style="31"/>
+    <col min="50" max="50" width="18.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="22.296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="8.8984375" style="31"/>
+    <col min="53" max="53" width="14.3984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.3984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="55" max="56" width="8.8984375" style="31"/>
+    <col min="57" max="57" width="12.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="22.69921875" style="31" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.8984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="20.09765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="8.8984375" style="31"/>
+    <col min="62" max="62" width="18.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="22.296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="8.8984375" style="31"/>
+    <col min="65" max="65" width="14.3984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="66" max="68" width="8.8984375" style="31"/>
+    <col min="69" max="69" width="12.59765625" style="31" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.69921875" style="31" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.8984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="16.59765625" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" ht="17.399999999999999">
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
       <c r="D1" s="29"/>
@@ -1167,7 +1165,7 @@
       <c r="W1" s="53"/>
       <c r="X1" s="54"/>
     </row>
-    <row r="2" spans="1:25" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="31.2">
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -1213,7 +1211,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" ht="27.6">
       <c r="B3" s="30"/>
       <c r="C3" s="30"/>
       <c r="D3" s="30"/>
@@ -1259,7 +1257,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" ht="17.399999999999999">
       <c r="B4" s="30"/>
       <c r="C4" s="30"/>
       <c r="D4" s="30"/>
@@ -1305,7 +1303,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" ht="27.6">
       <c r="A5" s="25"/>
       <c r="B5" s="30"/>
       <c r="C5" s="30"/>
@@ -1352,7 +1350,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" ht="27.6">
       <c r="A6" s="25"/>
       <c r="B6" s="30"/>
       <c r="C6" s="30"/>
@@ -1399,7 +1397,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" ht="18" thickBot="1">
       <c r="A7" s="25"/>
       <c r="B7" s="30"/>
       <c r="C7" s="30"/>
@@ -1446,7 +1444,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" ht="18" thickBot="1">
       <c r="A8" s="25"/>
       <c r="B8" s="30"/>
       <c r="C8" s="30"/>
@@ -1460,7 +1458,7 @@
       <c r="K8" s="30"/>
       <c r="L8" s="30"/>
     </row>
-    <row r="9" spans="1:25" ht="18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" ht="17.399999999999999">
       <c r="B9" s="30"/>
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
@@ -1486,7 +1484,7 @@
       <c r="W9" s="53"/>
       <c r="X9" s="54"/>
     </row>
-    <row r="10" spans="1:25" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" ht="31.2">
       <c r="B10" s="30"/>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
@@ -1532,7 +1530,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" ht="27.6">
       <c r="B11" s="30"/>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
@@ -1578,7 +1576,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25">
       <c r="N12" s="8" t="s">
         <v>31</v>
       </c>
@@ -1589,7 +1587,7 @@
         <v>14</v>
       </c>
       <c r="Q12" s="3">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="R12" s="3" t="s">
         <v>12</v>
@@ -1613,7 +1611,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25">
       <c r="N13" s="8" t="s">
         <v>32</v>
       </c>
@@ -1648,7 +1646,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" ht="27.6">
       <c r="N14" s="8" t="s">
         <v>33</v>
       </c>
@@ -1659,7 +1657,7 @@
         <v>14</v>
       </c>
       <c r="Q14" s="3">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="R14" s="3" t="s">
         <v>12</v>
@@ -1683,7 +1681,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25">
       <c r="B15" s="31"/>
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
@@ -1729,7 +1727,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:25" ht="14.4" thickBot="1">
       <c r="B16" s="31"/>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
@@ -1777,7 +1775,7 @@
       </c>
       <c r="Y16" s="36"/>
     </row>
-    <row r="17" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:26" ht="14.4" thickBot="1">
       <c r="B17" s="31"/>
       <c r="C17" s="31"/>
       <c r="D17" s="31"/>
@@ -1790,7 +1788,7 @@
       <c r="K17" s="31"/>
       <c r="L17" s="31"/>
     </row>
-    <row r="18" spans="2:26" ht="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:26" ht="17.399999999999999">
       <c r="B18" s="31"/>
       <c r="C18" s="31"/>
       <c r="D18" s="31"/>
@@ -1817,7 +1815,7 @@
       <c r="X18" s="54"/>
       <c r="Z18" s="37"/>
     </row>
-    <row r="19" spans="2:26" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:26" ht="31.2">
       <c r="B19" s="31"/>
       <c r="C19" s="31"/>
       <c r="D19" s="31"/>
@@ -1863,7 +1861,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="2:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:26" ht="27.6">
       <c r="B20" s="31"/>
       <c r="C20" s="31"/>
       <c r="D20" s="31"/>
@@ -1909,7 +1907,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:26">
       <c r="B21" s="31"/>
       <c r="C21" s="31"/>
       <c r="D21" s="31"/>
@@ -1931,7 +1929,7 @@
         <v>14</v>
       </c>
       <c r="Q21" s="3">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="R21" s="3" t="s">
         <v>12</v>
@@ -1955,7 +1953,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:26" ht="14.4" thickBot="1">
       <c r="B22" s="31"/>
       <c r="C22" s="31"/>
       <c r="D22" s="31"/>
@@ -2002,7 +2000,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:26">
       <c r="B23" s="31"/>
       <c r="C23" s="31"/>
       <c r="D23" s="31"/>
@@ -2015,7 +2013,7 @@
       <c r="K23" s="31"/>
       <c r="L23" s="31"/>
     </row>
-    <row r="24" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:26" ht="14.4" thickBot="1">
       <c r="B24" s="31"/>
       <c r="C24" s="31"/>
       <c r="D24" s="31"/>
@@ -2028,7 +2026,7 @@
       <c r="K24" s="31"/>
       <c r="L24" s="31"/>
     </row>
-    <row r="25" spans="2:26" ht="18" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:26" ht="17.399999999999999">
       <c r="B25" s="31"/>
       <c r="C25" s="31"/>
       <c r="D25" s="31"/>
@@ -2054,7 +2052,7 @@
       <c r="W25" s="53"/>
       <c r="X25" s="54"/>
     </row>
-    <row r="26" spans="2:26" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:26" ht="31.2">
       <c r="B26" s="31"/>
       <c r="C26" s="31"/>
       <c r="D26" s="31"/>
@@ -2100,7 +2098,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="2:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:26" ht="27.6">
       <c r="B27" s="31"/>
       <c r="C27" s="31"/>
       <c r="D27" s="31"/>
@@ -2146,7 +2144,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:26">
       <c r="B28" s="31"/>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -2192,7 +2190,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:26">
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
       <c r="D29" s="31"/>
@@ -2238,7 +2236,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:26" ht="14.4" thickBot="1">
       <c r="B30" s="31"/>
       <c r="C30" s="31"/>
       <c r="D30" s="31"/>
@@ -2284,7 +2282,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:26" ht="14.4" thickBot="1">
       <c r="B31" s="31"/>
       <c r="C31" s="31"/>
       <c r="D31" s="31"/>
@@ -2297,7 +2295,7 @@
       <c r="K31" s="31"/>
       <c r="L31" s="31"/>
     </row>
-    <row r="32" spans="2:26" ht="18" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:26" ht="17.399999999999999">
       <c r="B32" s="31"/>
       <c r="C32" s="31"/>
       <c r="D32" s="31"/>
@@ -2323,7 +2321,7 @@
       <c r="W32" s="53"/>
       <c r="X32" s="54"/>
     </row>
-    <row r="33" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:24" ht="31.2">
       <c r="B33" s="31"/>
       <c r="C33" s="31"/>
       <c r="D33" s="31"/>
@@ -2369,7 +2367,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="2:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:24" ht="22.2" customHeight="1">
       <c r="B34" s="31"/>
       <c r="C34" s="31"/>
       <c r="D34" s="31"/>
@@ -2415,7 +2413,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="35" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:24" ht="15">
       <c r="B35" s="31"/>
       <c r="C35" s="31"/>
       <c r="D35" s="31"/>
@@ -2461,7 +2459,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:24" ht="15">
       <c r="B36" s="31"/>
       <c r="C36" s="31"/>
       <c r="D36" s="31"/>
@@ -2507,7 +2505,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:24" ht="15">
       <c r="B37" s="31"/>
       <c r="C37" s="31"/>
       <c r="D37" s="31"/>
@@ -2553,7 +2551,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:24" ht="15">
       <c r="B38" s="31"/>
       <c r="C38" s="31"/>
       <c r="D38" s="31"/>
@@ -2599,7 +2597,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:24" ht="15">
       <c r="B39" s="31"/>
       <c r="C39" s="31"/>
       <c r="D39" s="31"/>
@@ -2645,7 +2643,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:24" ht="15">
       <c r="B40" s="31"/>
       <c r="C40" s="31"/>
       <c r="D40" s="31"/>
@@ -2691,7 +2689,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="2:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:24" ht="15.6" thickBot="1">
       <c r="B41" s="31"/>
       <c r="C41" s="31"/>
       <c r="D41" s="31"/>
@@ -2737,7 +2735,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:24" ht="14.4" thickBot="1">
       <c r="B42" s="31"/>
       <c r="C42" s="31"/>
       <c r="D42" s="31"/>
@@ -2750,7 +2748,7 @@
       <c r="K42" s="31"/>
       <c r="L42" s="31"/>
     </row>
-    <row r="43" spans="2:24" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:24" ht="18" thickBot="1">
       <c r="B43" s="31"/>
       <c r="C43" s="31"/>
       <c r="D43" s="31"/>
@@ -2776,7 +2774,7 @@
       <c r="W43" s="56"/>
       <c r="X43" s="57"/>
     </row>
-    <row r="44" spans="2:24" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:24" ht="31.8" thickBot="1">
       <c r="B44" s="31"/>
       <c r="C44" s="31"/>
       <c r="D44" s="31"/>
@@ -2822,7 +2820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:24">
       <c r="B45" s="31"/>
       <c r="C45" s="31"/>
       <c r="D45" s="31"/>
@@ -2868,7 +2866,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:24" ht="14.4" thickBot="1">
       <c r="B46" s="31"/>
       <c r="C46" s="31"/>
       <c r="D46" s="31"/>
@@ -2914,7 +2912,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:24" ht="14.4" thickBot="1">
       <c r="B47" s="31"/>
       <c r="C47" s="31"/>
       <c r="D47" s="31"/>
@@ -2938,7 +2936,7 @@
       <c r="W47" s="28"/>
       <c r="X47" s="50"/>
     </row>
-    <row r="48" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:24" ht="17.399999999999999">
       <c r="B48" s="31"/>
       <c r="C48" s="31"/>
       <c r="D48" s="31"/>
@@ -2964,7 +2962,7 @@
       <c r="W48" s="53"/>
       <c r="X48" s="54"/>
     </row>
-    <row r="49" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:24" ht="31.2">
       <c r="B49" s="31"/>
       <c r="C49" s="31"/>
       <c r="D49" s="31"/>
@@ -3010,7 +3008,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:24">
       <c r="B50" s="31"/>
       <c r="C50" s="31"/>
       <c r="D50" s="31"/>
@@ -3056,7 +3054,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="2:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:24" ht="14.4" thickBot="1">
       <c r="B51" s="31"/>
       <c r="C51" s="31"/>
       <c r="D51" s="31"/>
@@ -3102,7 +3100,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:24">
       <c r="B52" s="31"/>
       <c r="C52" s="31"/>
       <c r="D52" s="31"/>
@@ -3115,7 +3113,7 @@
       <c r="K52" s="31"/>
       <c r="L52" s="31"/>
     </row>
-    <row r="53" spans="2:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:24" ht="22.2" customHeight="1">
       <c r="B53" s="31"/>
       <c r="C53" s="31"/>
       <c r="D53" s="31"/>
@@ -3128,7 +3126,7 @@
       <c r="K53" s="31"/>
       <c r="L53" s="31"/>
     </row>
-    <row r="54" spans="2:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:24" ht="36" customHeight="1">
       <c r="B54" s="31"/>
       <c r="C54" s="31"/>
       <c r="D54" s="31"/>
@@ -3141,7 +3139,7 @@
       <c r="K54" s="31"/>
       <c r="L54" s="31"/>
     </row>
-    <row r="55" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:24" ht="42" customHeight="1">
       <c r="B55" s="31"/>
       <c r="C55" s="31"/>
       <c r="D55" s="31"/>
@@ -3154,7 +3152,7 @@
       <c r="K55" s="31"/>
       <c r="L55" s="31"/>
     </row>
-    <row r="56" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:24" ht="42" customHeight="1">
       <c r="B56" s="31"/>
       <c r="C56" s="31"/>
       <c r="D56" s="31"/>
@@ -3167,7 +3165,7 @@
       <c r="K56" s="31"/>
       <c r="L56" s="31"/>
     </row>
-    <row r="57" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:24" ht="42" customHeight="1">
       <c r="B57" s="31"/>
       <c r="C57" s="31"/>
       <c r="D57" s="31"/>
@@ -3180,7 +3178,7 @@
       <c r="K57" s="31"/>
       <c r="L57" s="31"/>
     </row>
-    <row r="58" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:24" ht="42" customHeight="1">
       <c r="B58" s="31"/>
       <c r="C58" s="31"/>
       <c r="D58" s="31"/>
@@ -3193,7 +3191,7 @@
       <c r="K58" s="31"/>
       <c r="L58" s="31"/>
     </row>
-    <row r="59" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:24" ht="42" customHeight="1">
       <c r="B59" s="31"/>
       <c r="C59" s="31"/>
       <c r="D59" s="31"/>
@@ -3206,7 +3204,7 @@
       <c r="K59" s="31"/>
       <c r="L59" s="31"/>
     </row>
-    <row r="60" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:24" ht="42" customHeight="1">
       <c r="B60" s="31"/>
       <c r="C60" s="31"/>
       <c r="D60" s="31"/>
@@ -3220,7 +3218,7 @@
       <c r="L60" s="31"/>
       <c r="M60" s="19"/>
     </row>
-    <row r="61" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:24" ht="42" customHeight="1">
       <c r="B61" s="31"/>
       <c r="C61" s="31"/>
       <c r="D61" s="31"/>
@@ -3233,7 +3231,7 @@
       <c r="K61" s="31"/>
       <c r="L61" s="31"/>
     </row>
-    <row r="62" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:24" ht="42" customHeight="1">
       <c r="B62" s="31"/>
       <c r="C62" s="31"/>
       <c r="D62" s="31"/>

</xml_diff>

<commit_message>
Alterando a documentação e o dicionário de dados - 22/04/2026
</commit_message>
<xml_diff>
--- a/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/dicionario_de_dados_projeto.xlsx
+++ b/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/dicionario_de_dados_projeto.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42db616d6e295501/Desktop/Códigos e Projetos/Projetos_ADS_Einstein/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B 789\Downloads\Projetos_ADSN_Einstein\Terceiro_Semestre\Projeto_Integrador\Documentação\dicionario_dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="166" documentId="13_ncr:1_{AF0911E6-20BD-4BF9-B7C3-EB184AF315FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D273743C-6F0F-47FC-9DC1-9D64D95543B0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{469F5BF7-1942-432A-8289-DDFBF75692AC}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="95">
   <si>
     <t>Mnemônico</t>
   </si>
@@ -323,13 +322,18 @@
   </si>
   <si>
     <t>"P"</t>
+  </si>
+  <si>
+    <t>DI - Diretor
+CO - Coordenador
+RT - Responsável de TI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -842,6 +846,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -858,15 +871,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1206,62 +1210,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{064BA25E-541B-4771-AFA8-C0176CB4D374}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:Z62"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.88671875" customWidth="1"/>
-    <col min="14" max="14" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.875" customWidth="1"/>
+    <col min="14" max="14" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.25" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.375" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="22" customWidth="1"/>
-    <col min="29" max="29" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="18.875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="22.375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="20.125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="22.375" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:24" ht="18">
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -1273,21 +1277,21 @@
       <c r="J1" s="25"/>
       <c r="K1" s="25"/>
       <c r="L1" s="25"/>
-      <c r="N1" s="57" t="s">
+      <c r="N1" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="58"/>
-      <c r="T1" s="58"/>
-      <c r="U1" s="58"/>
-      <c r="V1" s="58"/>
-      <c r="W1" s="58"/>
-      <c r="X1" s="59"/>
-    </row>
-    <row r="2" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O1" s="52"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="52"/>
+      <c r="V1" s="52"/>
+      <c r="W1" s="52"/>
+      <c r="X1" s="53"/>
+    </row>
+    <row r="2" spans="2:24" ht="31.5">
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
@@ -1333,7 +1337,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:24" ht="28.5">
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -1379,7 +1383,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:24" ht="18">
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
@@ -1425,7 +1429,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:24" ht="28.5">
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
@@ -1471,7 +1475,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:24" ht="28.5">
       <c r="B6" s="26"/>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -1517,7 +1521,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:24" ht="18">
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
@@ -1563,7 +1567,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:24" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:24" ht="29.25" thickBot="1">
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
@@ -1609,7 +1613,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="2:24" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:24" ht="18.75" thickBot="1">
       <c r="B9" s="26"/>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
@@ -1622,7 +1626,7 @@
       <c r="K9" s="26"/>
       <c r="L9" s="26"/>
     </row>
-    <row r="10" spans="2:24" ht="18" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:24" ht="18">
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -1634,21 +1638,21 @@
       <c r="J10" s="26"/>
       <c r="K10" s="26"/>
       <c r="L10" s="26"/>
-      <c r="N10" s="57" t="s">
+      <c r="N10" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="O10" s="58"/>
-      <c r="P10" s="58"/>
-      <c r="Q10" s="58"/>
-      <c r="R10" s="58"/>
-      <c r="S10" s="58"/>
-      <c r="T10" s="58"/>
-      <c r="U10" s="58"/>
-      <c r="V10" s="58"/>
-      <c r="W10" s="58"/>
-      <c r="X10" s="59"/>
-    </row>
-    <row r="11" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O10" s="52"/>
+      <c r="P10" s="52"/>
+      <c r="Q10" s="52"/>
+      <c r="R10" s="52"/>
+      <c r="S10" s="52"/>
+      <c r="T10" s="52"/>
+      <c r="U10" s="52"/>
+      <c r="V10" s="52"/>
+      <c r="W10" s="52"/>
+      <c r="X10" s="53"/>
+    </row>
+    <row r="11" spans="2:24" ht="31.5">
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -1694,7 +1698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:24" ht="28.5">
       <c r="N12" s="7" t="s">
         <v>24</v>
       </c>
@@ -1729,7 +1733,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:24">
       <c r="N13" s="7" t="s">
         <v>25</v>
       </c>
@@ -1764,7 +1768,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:24">
       <c r="N14" s="7" t="s">
         <v>26</v>
       </c>
@@ -1799,7 +1803,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:24">
       <c r="N15" s="7" t="s">
         <v>28</v>
       </c>
@@ -1834,7 +1838,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:24">
       <c r="N16" s="7" t="s">
         <v>62</v>
       </c>
@@ -1869,7 +1873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="13:26" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="13:26" ht="43.5" thickBot="1">
       <c r="N17" s="41" t="s">
         <v>27</v>
       </c>
@@ -1904,25 +1908,25 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="13:26" ht="15" thickBot="1">
       <c r="Z18" s="31"/>
     </row>
-    <row r="19" spans="13:26" ht="18" x14ac:dyDescent="0.3">
-      <c r="N19" s="51" t="s">
+    <row r="19" spans="13:26" ht="18">
+      <c r="N19" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="O19" s="52"/>
-      <c r="P19" s="52"/>
-      <c r="Q19" s="52"/>
-      <c r="R19" s="52"/>
-      <c r="S19" s="52"/>
-      <c r="T19" s="52"/>
-      <c r="U19" s="52"/>
-      <c r="V19" s="52"/>
-      <c r="W19" s="52"/>
-      <c r="X19" s="53"/>
-    </row>
-    <row r="20" spans="13:26" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O19" s="55"/>
+      <c r="P19" s="55"/>
+      <c r="Q19" s="55"/>
+      <c r="R19" s="55"/>
+      <c r="S19" s="55"/>
+      <c r="T19" s="55"/>
+      <c r="U19" s="55"/>
+      <c r="V19" s="55"/>
+      <c r="W19" s="55"/>
+      <c r="X19" s="56"/>
+    </row>
+    <row r="20" spans="13:26" ht="31.5">
       <c r="N20" s="29" t="s">
         <v>0</v>
       </c>
@@ -1957,7 +1961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="13:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="13:26" ht="28.5">
       <c r="N21" s="7" t="s">
         <v>76</v>
       </c>
@@ -1992,7 +1996,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="13:26" ht="72" thickBot="1">
       <c r="M22" s="32"/>
       <c r="N22" s="9" t="s">
         <v>77</v>
@@ -2024,27 +2028,27 @@
       <c r="W22" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="X22" s="21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="24" spans="13:26" ht="18" x14ac:dyDescent="0.3">
-      <c r="N24" s="51" t="s">
+      <c r="X22" s="49" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="13:26" ht="15" thickBot="1"/>
+    <row r="24" spans="13:26" ht="18">
+      <c r="N24" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="O24" s="52"/>
-      <c r="P24" s="52"/>
-      <c r="Q24" s="52"/>
-      <c r="R24" s="52"/>
-      <c r="S24" s="52"/>
-      <c r="T24" s="52"/>
-      <c r="U24" s="52"/>
-      <c r="V24" s="52"/>
-      <c r="W24" s="52"/>
-      <c r="X24" s="53"/>
-    </row>
-    <row r="25" spans="13:26" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O24" s="55"/>
+      <c r="P24" s="55"/>
+      <c r="Q24" s="55"/>
+      <c r="R24" s="55"/>
+      <c r="S24" s="55"/>
+      <c r="T24" s="55"/>
+      <c r="U24" s="55"/>
+      <c r="V24" s="55"/>
+      <c r="W24" s="55"/>
+      <c r="X24" s="56"/>
+    </row>
+    <row r="25" spans="13:26" ht="31.5">
       <c r="N25" s="29" t="s">
         <v>0</v>
       </c>
@@ -2079,7 +2083,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="13:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="13:26" ht="28.5">
       <c r="N26" s="7" t="s">
         <v>30</v>
       </c>
@@ -2114,7 +2118,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="13:26" x14ac:dyDescent="0.3">
+    <row r="27" spans="13:26">
       <c r="N27" s="7" t="s">
         <v>13</v>
       </c>
@@ -2149,7 +2153,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="13:26" ht="15" thickBot="1">
       <c r="N28" s="9" t="s">
         <v>31</v>
       </c>
@@ -2184,23 +2188,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="13:26" ht="18" x14ac:dyDescent="0.3">
-      <c r="N30" s="51" t="s">
+    <row r="29" spans="13:26" ht="15" thickBot="1"/>
+    <row r="30" spans="13:26" ht="18">
+      <c r="N30" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="O30" s="52"/>
-      <c r="P30" s="52"/>
-      <c r="Q30" s="52"/>
-      <c r="R30" s="52"/>
-      <c r="S30" s="52"/>
-      <c r="T30" s="52"/>
-      <c r="U30" s="52"/>
-      <c r="V30" s="52"/>
-      <c r="W30" s="52"/>
-      <c r="X30" s="53"/>
-    </row>
-    <row r="31" spans="13:26" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O30" s="55"/>
+      <c r="P30" s="55"/>
+      <c r="Q30" s="55"/>
+      <c r="R30" s="55"/>
+      <c r="S30" s="55"/>
+      <c r="T30" s="55"/>
+      <c r="U30" s="55"/>
+      <c r="V30" s="55"/>
+      <c r="W30" s="55"/>
+      <c r="X30" s="56"/>
+    </row>
+    <row r="31" spans="13:26" ht="31.5">
       <c r="N31" s="29" t="s">
         <v>0</v>
       </c>
@@ -2235,7 +2239,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="13:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="13:26" ht="28.5">
       <c r="N32" s="7" t="s">
         <v>33</v>
       </c>
@@ -2270,7 +2274,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="14:24" x14ac:dyDescent="0.3">
+    <row r="33" spans="14:24">
       <c r="N33" s="7" t="s">
         <v>65</v>
       </c>
@@ -2305,7 +2309,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="14:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="14:24" ht="22.15" customHeight="1">
       <c r="N34" s="7" t="s">
         <v>24</v>
       </c>
@@ -2340,7 +2344,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="14:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="14:24" ht="15" thickBot="1">
       <c r="N35" s="9" t="s">
         <v>36</v>
       </c>
@@ -2375,23 +2379,23 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="14:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="37" spans="14:24" ht="18" x14ac:dyDescent="0.3">
-      <c r="N37" s="51" t="s">
+    <row r="36" spans="14:24" ht="15" thickBot="1"/>
+    <row r="37" spans="14:24" ht="18">
+      <c r="N37" s="54" t="s">
         <v>42</v>
       </c>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
-      <c r="R37" s="52"/>
-      <c r="S37" s="52"/>
-      <c r="T37" s="52"/>
-      <c r="U37" s="52"/>
-      <c r="V37" s="52"/>
-      <c r="W37" s="52"/>
-      <c r="X37" s="53"/>
-    </row>
-    <row r="38" spans="14:24" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O37" s="55"/>
+      <c r="P37" s="55"/>
+      <c r="Q37" s="55"/>
+      <c r="R37" s="55"/>
+      <c r="S37" s="55"/>
+      <c r="T37" s="55"/>
+      <c r="U37" s="55"/>
+      <c r="V37" s="55"/>
+      <c r="W37" s="55"/>
+      <c r="X37" s="56"/>
+    </row>
+    <row r="38" spans="14:24" ht="31.5">
       <c r="N38" s="29" t="s">
         <v>0</v>
       </c>
@@ -2426,7 +2430,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="14:24" ht="15">
       <c r="N39" s="34" t="s">
         <v>43</v>
       </c>
@@ -2461,7 +2465,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="14:24" ht="15">
       <c r="N40" s="34" t="s">
         <v>44</v>
       </c>
@@ -2496,7 +2500,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="14:24" ht="15">
       <c r="N41" s="34" t="s">
         <v>34</v>
       </c>
@@ -2531,7 +2535,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="14:24" ht="15">
       <c r="N42" s="34" t="s">
         <v>35</v>
       </c>
@@ -2566,7 +2570,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="14:24" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="14:24" ht="45">
       <c r="N43" s="34" t="s">
         <v>45</v>
       </c>
@@ -2601,7 +2605,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="14:24" ht="15">
       <c r="N44" s="34" t="s">
         <v>33</v>
       </c>
@@ -2636,7 +2640,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="14:24" ht="15">
       <c r="N45" s="34" t="s">
         <v>18</v>
       </c>
@@ -2671,7 +2675,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="14:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="14:24" ht="15.75" thickBot="1">
       <c r="N46" s="35" t="s">
         <v>24</v>
       </c>
@@ -2706,23 +2710,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="14:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="48" spans="14:24" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="N48" s="54" t="s">
+    <row r="47" spans="14:24" ht="15" thickBot="1"/>
+    <row r="48" spans="14:24" ht="18.75" thickBot="1">
+      <c r="N48" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="O48" s="55"/>
-      <c r="P48" s="55"/>
-      <c r="Q48" s="55"/>
-      <c r="R48" s="55"/>
-      <c r="S48" s="55"/>
-      <c r="T48" s="55"/>
-      <c r="U48" s="55"/>
-      <c r="V48" s="55"/>
-      <c r="W48" s="55"/>
-      <c r="X48" s="56"/>
-    </row>
-    <row r="49" spans="13:24" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O48" s="58"/>
+      <c r="P48" s="58"/>
+      <c r="Q48" s="58"/>
+      <c r="R48" s="58"/>
+      <c r="S48" s="58"/>
+      <c r="T48" s="58"/>
+      <c r="U48" s="58"/>
+      <c r="V48" s="58"/>
+      <c r="W48" s="58"/>
+      <c r="X48" s="59"/>
+    </row>
+    <row r="49" spans="13:24" ht="32.25" thickBot="1">
       <c r="N49" s="1" t="s">
         <v>0</v>
       </c>
@@ -2757,7 +2761,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="13:24" x14ac:dyDescent="0.3">
+    <row r="50" spans="13:24">
       <c r="N50" s="5" t="s">
         <v>30</v>
       </c>
@@ -2792,7 +2796,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="13:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="13:24" ht="15" thickBot="1">
       <c r="N51" s="9" t="s">
         <v>18</v>
       </c>
@@ -2827,7 +2831,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="13:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="13:24" ht="15" thickBot="1">
       <c r="N52" s="17"/>
       <c r="O52" s="23"/>
       <c r="P52" s="17"/>
@@ -2840,22 +2844,22 @@
       <c r="W52" s="24"/>
       <c r="X52" s="39"/>
     </row>
-    <row r="53" spans="13:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="N53" s="51" t="s">
+    <row r="53" spans="13:24" ht="22.15" customHeight="1">
+      <c r="N53" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="O53" s="52"/>
-      <c r="P53" s="52"/>
-      <c r="Q53" s="52"/>
-      <c r="R53" s="52"/>
-      <c r="S53" s="52"/>
-      <c r="T53" s="52"/>
-      <c r="U53" s="52"/>
-      <c r="V53" s="52"/>
-      <c r="W53" s="52"/>
-      <c r="X53" s="53"/>
-    </row>
-    <row r="54" spans="13:24" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="O53" s="55"/>
+      <c r="P53" s="55"/>
+      <c r="Q53" s="55"/>
+      <c r="R53" s="55"/>
+      <c r="S53" s="55"/>
+      <c r="T53" s="55"/>
+      <c r="U53" s="55"/>
+      <c r="V53" s="55"/>
+      <c r="W53" s="55"/>
+      <c r="X53" s="56"/>
+    </row>
+    <row r="54" spans="13:24" ht="31.5">
       <c r="N54" s="29" t="s">
         <v>0</v>
       </c>
@@ -2890,7 +2894,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="13:24" x14ac:dyDescent="0.3">
+    <row r="55" spans="13:24">
       <c r="N55" s="7" t="s">
         <v>30</v>
       </c>
@@ -2925,7 +2929,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="13:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="13:24" ht="15" thickBot="1">
       <c r="N56" s="9" t="s">
         <v>33</v>
       </c>
@@ -2960,14 +2964,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="13:24" ht="42" customHeight="1"/>
+    <row r="58" spans="13:24" ht="42" customHeight="1"/>
+    <row r="59" spans="13:24" ht="42" customHeight="1"/>
+    <row r="60" spans="13:24" ht="42" customHeight="1">
       <c r="M60" s="17"/>
     </row>
-    <row r="61" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="13:24" ht="42" customHeight="1"/>
+    <row r="62" spans="13:24" ht="42" customHeight="1"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="N1:X1"/>

</xml_diff>

<commit_message>
Atualizando a documentação (prazo final para entrega: 26/04/2026) - 25/04/2026
</commit_message>
<xml_diff>
--- a/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/dicionario_de_dados_projeto.xlsx
+++ b/Terceiro_Semestre/Projeto_Integrador/Documentação/dicionario_dados/dicionario_de_dados_projeto.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B 789\Downloads\Projetos_ADSN_Einstein\Terceiro_Semestre\Projeto_Integrador\Documentação\dicionario_dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42db616d6e295501/Desktop/Códigos e Projetos/Projetos_ADS_Einstein/Terceiro_Semestre/Projeto_Integrador/Documentação/Dicionario_dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_03EE63304EB3ECF35CAEC07740CEC154711758A2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7CCB397-6C45-437C-87E4-2494872E7B98}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -19,15 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -332,8 +324,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -364,6 +356,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -694,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -871,6 +871,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -888,10 +891,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1210,62 +1209,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:Z62"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.875" customWidth="1"/>
-    <col min="14" max="14" width="21.375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" customWidth="1"/>
+    <col min="14" max="14" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="4.625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="25.125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.25" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="22" customWidth="1"/>
-    <col min="29" max="29" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="22.625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="18.875" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="22.625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="20.125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.625" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="19.875" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="16.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" ht="18">
+    <row r="1" spans="2:24" ht="18" x14ac:dyDescent="0.3">
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
@@ -1291,7 +1290,7 @@
       <c r="W1" s="52"/>
       <c r="X1" s="53"/>
     </row>
-    <row r="2" spans="2:24" ht="31.5">
+    <row r="2" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
@@ -1337,7 +1336,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="2:24" ht="28.5">
+    <row r="3" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -1383,7 +1382,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="2:24" ht="18">
+    <row r="4" spans="2:24" ht="18" x14ac:dyDescent="0.3">
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
@@ -1429,7 +1428,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:24" ht="28.5">
+    <row r="5" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
@@ -1475,7 +1474,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="2:24" ht="28.5">
+    <row r="6" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B6" s="26"/>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
@@ -1521,7 +1520,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="2:24" ht="18">
+    <row r="7" spans="2:24" ht="18" x14ac:dyDescent="0.3">
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
@@ -1567,7 +1566,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:24" ht="29.25" thickBot="1">
+    <row r="8" spans="2:24" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
@@ -1613,7 +1612,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="2:24" ht="18.75" thickBot="1">
+    <row r="9" spans="2:24" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="26"/>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
@@ -1626,7 +1625,7 @@
       <c r="K9" s="26"/>
       <c r="L9" s="26"/>
     </row>
-    <row r="10" spans="2:24" ht="18">
+    <row r="10" spans="2:24" ht="18" x14ac:dyDescent="0.3">
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -1652,7 +1651,7 @@
       <c r="W10" s="52"/>
       <c r="X10" s="53"/>
     </row>
-    <row r="11" spans="2:24" ht="31.5">
+    <row r="11" spans="2:24" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
@@ -1698,7 +1697,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:24" ht="28.5">
+    <row r="12" spans="2:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="N12" s="7" t="s">
         <v>24</v>
       </c>
@@ -1733,7 +1732,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="2:24">
+    <row r="13" spans="2:24" x14ac:dyDescent="0.3">
       <c r="N13" s="7" t="s">
         <v>25</v>
       </c>
@@ -1768,7 +1767,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="2:24">
+    <row r="14" spans="2:24" x14ac:dyDescent="0.3">
       <c r="N14" s="7" t="s">
         <v>26</v>
       </c>
@@ -1803,7 +1802,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="2:24">
+    <row r="15" spans="2:24" x14ac:dyDescent="0.3">
       <c r="N15" s="7" t="s">
         <v>28</v>
       </c>
@@ -1838,7 +1837,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="2:24">
+    <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="N16" s="7" t="s">
         <v>62</v>
       </c>
@@ -1846,7 +1845,7 @@
         <v>63</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="Q16" s="3">
         <v>10</v>
@@ -1873,7 +1872,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="13:26" ht="43.5" thickBot="1">
+    <row r="17" spans="13:26" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N17" s="41" t="s">
         <v>27</v>
       </c>
@@ -1889,7 +1888,7 @@
       <c r="R17" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="S17" s="42" t="s">
+      <c r="S17" s="60" t="s">
         <v>12</v>
       </c>
       <c r="T17" s="42" t="s">
@@ -1908,10 +1907,10 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="13:26" ht="15" thickBot="1">
+    <row r="18" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="Z18" s="31"/>
     </row>
-    <row r="19" spans="13:26" ht="18">
+    <row r="19" spans="13:26" ht="18" x14ac:dyDescent="0.3">
       <c r="N19" s="54" t="s">
         <v>75</v>
       </c>
@@ -1926,7 +1925,7 @@
       <c r="W19" s="55"/>
       <c r="X19" s="56"/>
     </row>
-    <row r="20" spans="13:26" ht="31.5">
+    <row r="20" spans="13:26" ht="31.2" x14ac:dyDescent="0.3">
       <c r="N20" s="29" t="s">
         <v>0</v>
       </c>
@@ -1961,7 +1960,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="13:26" ht="28.5">
+    <row r="21" spans="13:26" ht="28.8" x14ac:dyDescent="0.3">
       <c r="N21" s="7" t="s">
         <v>76</v>
       </c>
@@ -1996,7 +1995,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="13:26" ht="72" thickBot="1">
+    <row r="22" spans="13:26" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="M22" s="32"/>
       <c r="N22" s="9" t="s">
         <v>77</v>
@@ -2032,8 +2031,8 @@
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="13:26" ht="15" thickBot="1"/>
-    <row r="24" spans="13:26" ht="18">
+    <row r="23" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="13:26" ht="18" x14ac:dyDescent="0.3">
       <c r="N24" s="54" t="s">
         <v>29</v>
       </c>
@@ -2048,7 +2047,7 @@
       <c r="W24" s="55"/>
       <c r="X24" s="56"/>
     </row>
-    <row r="25" spans="13:26" ht="31.5">
+    <row r="25" spans="13:26" ht="31.2" x14ac:dyDescent="0.3">
       <c r="N25" s="29" t="s">
         <v>0</v>
       </c>
@@ -2083,7 +2082,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="13:26" ht="28.5">
+    <row r="26" spans="13:26" ht="28.8" x14ac:dyDescent="0.3">
       <c r="N26" s="7" t="s">
         <v>30</v>
       </c>
@@ -2118,7 +2117,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="13:26">
+    <row r="27" spans="13:26" x14ac:dyDescent="0.3">
       <c r="N27" s="7" t="s">
         <v>13</v>
       </c>
@@ -2153,7 +2152,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="13:26" ht="15" thickBot="1">
+    <row r="28" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N28" s="9" t="s">
         <v>31</v>
       </c>
@@ -2188,8 +2187,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="13:26" ht="15" thickBot="1"/>
-    <row r="30" spans="13:26" ht="18">
+    <row r="29" spans="13:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="13:26" ht="18" x14ac:dyDescent="0.3">
       <c r="N30" s="54" t="s">
         <v>32</v>
       </c>
@@ -2204,7 +2203,7 @@
       <c r="W30" s="55"/>
       <c r="X30" s="56"/>
     </row>
-    <row r="31" spans="13:26" ht="31.5">
+    <row r="31" spans="13:26" ht="31.2" x14ac:dyDescent="0.3">
       <c r="N31" s="29" t="s">
         <v>0</v>
       </c>
@@ -2239,7 +2238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="13:26" ht="28.5">
+    <row r="32" spans="13:26" ht="28.8" x14ac:dyDescent="0.3">
       <c r="N32" s="7" t="s">
         <v>33</v>
       </c>
@@ -2274,7 +2273,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="14:24">
+    <row r="33" spans="14:24" x14ac:dyDescent="0.3">
       <c r="N33" s="7" t="s">
         <v>65</v>
       </c>
@@ -2309,7 +2308,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="14:24" ht="22.15" customHeight="1">
+    <row r="34" spans="14:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="N34" s="7" t="s">
         <v>24</v>
       </c>
@@ -2344,7 +2343,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="14:24" ht="15" thickBot="1">
+    <row r="35" spans="14:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N35" s="9" t="s">
         <v>36</v>
       </c>
@@ -2379,8 +2378,8 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="14:24" ht="15" thickBot="1"/>
-    <row r="37" spans="14:24" ht="18">
+    <row r="36" spans="14:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="37" spans="14:24" ht="18" x14ac:dyDescent="0.3">
       <c r="N37" s="54" t="s">
         <v>42</v>
       </c>
@@ -2395,7 +2394,7 @@
       <c r="W37" s="55"/>
       <c r="X37" s="56"/>
     </row>
-    <row r="38" spans="14:24" ht="31.5">
+    <row r="38" spans="14:24" ht="31.2" x14ac:dyDescent="0.3">
       <c r="N38" s="29" t="s">
         <v>0</v>
       </c>
@@ -2430,7 +2429,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="14:24" ht="15">
+    <row r="39" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="N39" s="34" t="s">
         <v>43</v>
       </c>
@@ -2465,7 +2464,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="14:24" ht="15">
+    <row r="40" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="N40" s="34" t="s">
         <v>44</v>
       </c>
@@ -2500,7 +2499,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="14:24" ht="15">
+    <row r="41" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="N41" s="34" t="s">
         <v>34</v>
       </c>
@@ -2535,7 +2534,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="14:24" ht="15">
+    <row r="42" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="N42" s="34" t="s">
         <v>35</v>
       </c>
@@ -2570,7 +2569,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="14:24" ht="45">
+    <row r="43" spans="14:24" ht="46.8" x14ac:dyDescent="0.3">
       <c r="N43" s="34" t="s">
         <v>45</v>
       </c>
@@ -2605,7 +2604,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="14:24" ht="15">
+    <row r="44" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="N44" s="34" t="s">
         <v>33</v>
       </c>
@@ -2640,7 +2639,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="14:24" ht="15">
+    <row r="45" spans="14:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="N45" s="34" t="s">
         <v>18</v>
       </c>
@@ -2675,7 +2674,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="14:24" ht="15.75" thickBot="1">
+    <row r="46" spans="14:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N46" s="35" t="s">
         <v>24</v>
       </c>
@@ -2710,8 +2709,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="14:24" ht="15" thickBot="1"/>
-    <row r="48" spans="14:24" ht="18.75" thickBot="1">
+    <row r="47" spans="14:24" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="14:24" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N48" s="57" t="s">
         <v>56</v>
       </c>
@@ -2726,7 +2725,7 @@
       <c r="W48" s="58"/>
       <c r="X48" s="59"/>
     </row>
-    <row r="49" spans="13:24" ht="32.25" thickBot="1">
+    <row r="49" spans="13:24" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N49" s="1" t="s">
         <v>0</v>
       </c>
@@ -2761,7 +2760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="13:24">
+    <row r="50" spans="13:24" x14ac:dyDescent="0.3">
       <c r="N50" s="5" t="s">
         <v>30</v>
       </c>
@@ -2796,7 +2795,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="13:24" ht="15" thickBot="1">
+    <row r="51" spans="13:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N51" s="9" t="s">
         <v>18</v>
       </c>
@@ -2831,7 +2830,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="13:24" ht="15" thickBot="1">
+    <row r="52" spans="13:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N52" s="17"/>
       <c r="O52" s="23"/>
       <c r="P52" s="17"/>
@@ -2844,7 +2843,7 @@
       <c r="W52" s="24"/>
       <c r="X52" s="39"/>
     </row>
-    <row r="53" spans="13:24" ht="22.15" customHeight="1">
+    <row r="53" spans="13:24" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="N53" s="54" t="s">
         <v>58</v>
       </c>
@@ -2859,7 +2858,7 @@
       <c r="W53" s="55"/>
       <c r="X53" s="56"/>
     </row>
-    <row r="54" spans="13:24" ht="31.5">
+    <row r="54" spans="13:24" ht="31.2" x14ac:dyDescent="0.3">
       <c r="N54" s="29" t="s">
         <v>0</v>
       </c>
@@ -2894,7 +2893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="13:24">
+    <row r="55" spans="13:24" x14ac:dyDescent="0.3">
       <c r="N55" s="7" t="s">
         <v>30</v>
       </c>
@@ -2929,7 +2928,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="13:24" ht="15" thickBot="1">
+    <row r="56" spans="13:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="N56" s="9" t="s">
         <v>33</v>
       </c>
@@ -2964,14 +2963,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="13:24" ht="42" customHeight="1"/>
-    <row r="58" spans="13:24" ht="42" customHeight="1"/>
-    <row r="59" spans="13:24" ht="42" customHeight="1"/>
-    <row r="60" spans="13:24" ht="42" customHeight="1">
+    <row r="57" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M60" s="17"/>
     </row>
-    <row r="61" spans="13:24" ht="42" customHeight="1"/>
-    <row r="62" spans="13:24" ht="42" customHeight="1"/>
+    <row r="61" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="13:24" ht="42" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="N1:X1"/>

</xml_diff>